<commit_message>
Updated ai audit log with 2 rows
</commit_message>
<xml_diff>
--- a/AI Audit Log_DangXuanThong.xlsx
+++ b/AI Audit Log_DangXuanThong.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
     <t>STT</t>
   </si>
@@ -40,19 +40,54 @@
   </si>
   <si>
     <t xml:space="preserve">Human Delta &amp; Reflection</t>
+  </si>
+  <si>
+    <t>DECISION</t>
+  </si>
+  <si>
+    <t>Abstraction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thiết kế database cho hệ thống multi-branch spa</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Đề xuất các entity quan trọng cho hệ thống quản lý spa nhiều chi nhánh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI đề xuất các bảng Users, Branches, Services, Employees, Bookings, BookingSlots, Reviews và RevenueReports</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Điều chỉnh thêm branch_id ở nhiều bảng để phù hợp mô hình đa chi nhánh
+- Tách BookingSlots riêng thay vì lưu trực tiếp trong Bookings để dễ quản lý slot động</t>
   </si>
   <si>
     <t xml:space="preserve">• Critical Thinking: AI đúng/sai ở đâu? Phát hiện hallucination?
 • Contextualization: Bối cảnh thực tế mà AI không biết?
 • Creative Synthesis: Tôi đã thay đổi/kết hợp/tối ưu như thế nào?
 • Decision Ownership: Quyết định cuối cùng và lý do?</t>
+  </si>
+  <si>
+    <t>Algorithms</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thiết kế flow booking cho khách hàng.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mô tả quy trình booking phù hợp cho hệ thống spa nhiều chi nhánh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">AI đề xuất flow gồm chọn dịch vụ → tìm branch gần nhất → kiểm tra slot → booking hoặc suggest branch khác</t>
+  </si>
+  <si>
+    <t xml:space="preserve">- Giữ nguyên flow chính vì phù hợp với yêu cầu thực tế
+- Bổ sung chức năng xem lịch sử booking và đánh giá nhân viên sau khi hoàn thành dịch vụ</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11.000000"/>
       <color theme="1"/>
@@ -68,8 +103,12 @@
     </font>
     <font>
       <sz val="12.000000"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="11.000000"/>
       <color indexed="64"/>
-      <name val="Times New Roman"/>
+      <name val="Open Sans"/>
     </font>
   </fonts>
   <fills count="2">
@@ -107,29 +146,46 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="14">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf fontId="1" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
+      <alignment horizontal="justify" vertical="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="1" numFmtId="49" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -650,140 +706,170 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
   <sheetFormatPr defaultRowHeight="16.5"/>
   <cols>
-    <col bestFit="1" customWidth="1" min="1" max="1" width="3.82421875"/>
-    <col customWidth="1" min="2" max="2" width="13.625"/>
-    <col customWidth="1" min="3" max="3" width="26.25390625"/>
-    <col customWidth="1" min="4" max="4" width="15.375"/>
-    <col customWidth="1" min="5" max="5" width="31.625"/>
-    <col customWidth="1" min="6" max="6" width="12.75390625"/>
-    <col customWidth="1" min="7" max="7" width="50.50390625"/>
+    <col bestFit="1" customWidth="1" min="1" max="1" style="1" width="3.82421875"/>
+    <col customWidth="1" min="2" max="2" style="1" width="13.625"/>
+    <col bestFit="1" customWidth="1" min="3" max="3" style="1" width="25.32421875"/>
+    <col customWidth="1" min="4" max="4" style="1" width="43.75390625"/>
+    <col customWidth="1" min="5" max="5" style="2" width="31.625"/>
+    <col customWidth="1" min="6" max="6" style="2" width="37.875"/>
+    <col customWidth="1" min="7" max="7" style="2" width="50.50390625"/>
+    <col customWidth="1" min="8" max="8" style="1" width="62.625"/>
+    <col min="9" max="9" style="1" width="9.00390625"/>
+    <col min="10" max="16384" style="1" width="9.00390625"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="4" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" ht="99">
-      <c r="A2" s="2">
+    <row r="2" ht="66">
+      <c r="A2" s="5">
         <v>1</v>
       </c>
-      <c r="B2" s="2"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="6" t="s">
+      <c r="B2" s="5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="3" ht="18">
-      <c r="A3" s="7"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
+      <c r="C2" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="H2" s="9" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="3" ht="49.5">
+      <c r="A3" s="5">
+        <v>2</v>
+      </c>
+      <c r="B3" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="F3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="G3" s="12" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="4" ht="18">
-      <c r="A4" s="7"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7"/>
-      <c r="G4" s="7"/>
+      <c r="A4" s="5"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="10"/>
+      <c r="D4" s="10"/>
+      <c r="E4" s="13"/>
+      <c r="F4" s="13"/>
+      <c r="G4" s="13"/>
     </row>
     <row r="5" ht="18">
-      <c r="A5" s="7"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
+      <c r="A5" s="5"/>
+      <c r="B5" s="5"/>
+      <c r="C5" s="10"/>
+      <c r="D5" s="10"/>
+      <c r="E5" s="13"/>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13"/>
     </row>
     <row r="6" ht="16.5">
-      <c r="A6" s="7"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7"/>
-      <c r="E6" s="7"/>
-      <c r="F6" s="7"/>
-      <c r="G6" s="7"/>
+      <c r="A6" s="5"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
     </row>
     <row r="7" ht="16.5">
-      <c r="A7" s="7"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-      <c r="F7" s="7"/>
-      <c r="G7" s="7"/>
+      <c r="A7" s="5"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="5"/>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
     </row>
     <row r="8" ht="16.5">
-      <c r="A8" s="7"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-      <c r="F8" s="7"/>
-      <c r="G8" s="7"/>
+      <c r="A8" s="5"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="13"/>
     </row>
     <row r="9" ht="16.5">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
+      <c r="A9" s="5"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
     </row>
     <row r="10" ht="16.5">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
+      <c r="A10" s="5"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
     </row>
     <row r="11" ht="16.5">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
+      <c r="A11" s="5"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
     </row>
     <row r="12" ht="16.5">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
+      <c r="A12" s="5"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="13"/>
+      <c r="F12" s="13"/>
+      <c r="G12" s="13"/>
     </row>
   </sheetData>
   <printOptions headings="0" gridLines="0"/>
@@ -793,25 +879,25 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="4" disablePrompts="0">
-        <x14:dataValidation xr:uid="{001200D3-00D3-4D8B-8396-00070001008A}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" prompt="" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00930072-001D-4ACC-9B74-00DB00FF00E1}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" prompt="" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>"DECISION,PROBLEM-SOLVING,VERIFICATION"</xm:f>
           </x14:formula1>
           <xm:sqref>B2:B1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00EF0063-0056-48C1-97FB-007F000600D9}" type="none" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" prompt="" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00080053-00DB-42F1-8DB0-00E2003E005A}" type="none" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" prompt="" promptTitle="" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>"DECISION,PROBLEM-SOLVING,VERIFICATION"</xm:f>
           </x14:formula1>
           <xm:sqref>B1</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{00D30060-0060-4B20-98C4-006A00670063}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00C80009-00E7-428E-8FD7-0090002E0035}" type="list" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>"Decomposition,Pattern Recognition,Abstraction,Algorithms,Research stage"</xm:f>
           </x14:formula1>
           <xm:sqref>C2:C1048576</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation xr:uid="{007900B7-00E5-4FEE-934B-001000B800EE}" type="none" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
+        <x14:dataValidation xr:uid="{00CE00C8-0065-49ED-8B5B-00CB006A00CC}" type="none" allowBlank="1" errorStyle="stop" imeMode="noControl" operator="between" showDropDown="0" showErrorMessage="1" showInputMessage="1">
           <x14:formula1>
             <xm:f>"Decomposition,Pattern Recognition,Abstraction,Algorithms,Research stage"</xm:f>
           </x14:formula1>

</xml_diff>